<commit_message>
Completed Milestone 2- Build Code Analysis Agent, Build Security Vulnerability Agent, Implement multi-agent orchestration, Validate agent detection accuracy
</commit_message>
<xml_diff>
--- a/agile_documents/Defect_Tracker Template_v0.1.xlsx
+++ b/agile_documents/Defect_Tracker Template_v0.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3DF93A8BBD052DAA/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3df93a8bbd052daa/Desktop/Milestone 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{EC4EACBB-8F7A-4584-8E39-BBE80DB3A2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FAB3497-6B10-4C9E-9347-8CF239DFD978}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{EC4EACBB-8F7A-4584-8E39-BBE80DB3A2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17ED926C-2465-4F53-B046-04E9CAE093DF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Sl No</t>
   </si>
@@ -87,6 +87,35 @@
   </si>
   <si>
     <t>All import errors, missing paths, and deprecation warnings have been fully resolved; the RAG knowledge base runs efficiently and renders unique search results seamlessly.</t>
+  </si>
+  <si>
+    <t>Overlapping regex patterns between security and quality agents resulted in duplicate finding cards appearing on the same line.</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Implemented advanced line-grouping logic and severity merging inside </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>workflow.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to unify multi-agent issues cleanly.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verified that all multi-agent findings now render uniquely with prioritized high severities per line.</t>
   </si>
 </sst>
 </file>
@@ -196,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -229,8 +258,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -247,6 +279,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -621,18 +657,40 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="12"/>
+    <row r="3" spans="1:11" ht="79.2">
+      <c r="A3" s="4">
+        <v>3</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="5">
+        <v>46323</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="5">
+        <v>46320</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="13" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:11" ht="15.6">
       <c r="A4" s="4"/>
@@ -1044,18 +1102,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1077,18 +1135,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>